<commit_message>
Regenerate Examples for Tests
Fixed Dateformat to be same on every platform
</commit_message>
<xml_diff>
--- a/XlsxSharp.Tests/Resource/Examples/PageSetup/HeaderFooters.xlsx
+++ b/XlsxSharp.Tests/Resource/Examples/PageSetup/HeaderFooters.xlsx
@@ -361,11 +361,11 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter differentOddEven="1" differentFirst="1" scaleWithDoc="0" alignWithMargins="0">
-    <x:oddHeader>&amp;LCreated with ClosedXML</x:oddHeader>
+    <x:oddHeader>&amp;LCreated with XlsxSharp</x:oddHeader>
     <x:oddFooter>&amp;C&amp;P / &amp;N&amp;R&amp;Z&amp;F</x:oddFooter>
-    <x:evenHeader>&amp;LCreated with ClosedXML</x:evenHeader>
+    <x:evenHeader>&amp;LCreated with XlsxSharp</x:evenHeader>
     <x:evenFooter>&amp;C&amp;P / &amp;N</x:evenFooter>
-    <x:firstHeader>&amp;LCreated with ClosedXML&amp;R&amp;"-,Bold"The &amp;"-,Regular"&amp;KFF0000First &amp;"-,Regular"&amp;E&amp;K0000FFColorful &amp;E&amp;"Broadway,Bold Italic"&amp;K000000Page</x:firstHeader>
+    <x:firstHeader>&amp;LCreated with XlsxSharp&amp;R&amp;"-,Bold"The &amp;"-,Regular"&amp;KFF0000First &amp;"-,Regular"&amp;E&amp;K0000FFColorful &amp;E&amp;"Broadway,Bold Italic"&amp;K000000Page</x:firstHeader>
     <x:firstFooter>&amp;C&amp;P / &amp;N</x:firstFooter>
   </x:headerFooter>
   <x:tableParts count="0"/>

</xml_diff>